<commit_message>
Rebrand frontend as Compvd.ai
</commit_message>
<xml_diff>
--- a/spectramind/public/templates/employee-import-template.xlsx
+++ b/spectramind/public/templates/employee-import-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" r:id="R1b3473ca181f4037"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R08f497f0e1d64f4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" r:id="R70388807471b44e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R2d4b78de6e41431e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -450,7 +450,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6facff6838834b44"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1666e3a9f3de403c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -467,7 +467,7 @@
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
       <x:c r="A1" s="9" t="str">
-        <x:v>SpectraMind Employee Import Template</x:v>
+        <x:v>compvd Employee Import Template</x:v>
       </x:c>
       <x:c r="B1" s="9"/>
       <x:c r="C1" s="9"/>

</xml_diff>